<commit_message>
finalizacion wip de la libreria procesadora de tramas modbus, todavia requiere comprobaciones por lo que no esta implementada por completo, se agregaran tests posteriomente. Se agrego LICENSE para indicar la propiedad intelectual del repositorio, se da espacio para contactar en caso de interes del codigo, y tambien seagrego un readme para explicar mas sobre el proposito general del codigo
</commit_message>
<xml_diff>
--- a/modbus.xlsx
+++ b/modbus.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\windows\projects\rust\firerust\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{220D2CD7-325A-448B-8EA4-C4172A2CA27C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75D2BCEE-3635-4434-8019-C151879B9C84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="70">
   <si>
     <t>MODBUS INSTRUCTION SAMPLE</t>
   </si>
@@ -197,9 +197,6 @@
     <t>write_multiple_coils</t>
   </si>
   <si>
-    <t>[ 5 ]</t>
-  </si>
-  <si>
     <t>7E</t>
   </si>
   <si>
@@ -242,9 +239,6 @@
     <t>4,5</t>
   </si>
   <si>
-    <t>01 0F 00 0A 00 0C 02 53 05 19 E9</t>
-  </si>
-  <si>
     <t>01 10 00 0A 00 03 06 00 0A 00 0B 00 0C 2F 66</t>
   </si>
   <si>
@@ -252,17 +246,36 @@
   </si>
   <si>
     <t>(7, 8)..Max-2</t>
+  </si>
+  <si>
+    <t>01 0F 00 0A 00 0C 02 FF 0F E4 EE</t>
+  </si>
+  <si>
+    <t>[ 255 15 ]</t>
+  </si>
+  <si>
+    <t>pos 6 7</t>
+  </si>
+  <si>
+    <t>pos 8 9</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -283,7 +296,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -311,12 +324,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="2"/>
-        <bgColor indexed="2"/>
       </patternFill>
     </fill>
   </fills>
@@ -349,24 +356,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -627,56 +634,56 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:28" ht="30" customHeight="1">
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="13"/>
-      <c r="F2" s="14" t="s">
+      <c r="E2" s="15"/>
+      <c r="F2" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="G2" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="14" t="s">
+      <c r="H2" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="15" t="s">
+      <c r="I2" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="14" t="s">
+      <c r="J2" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="K2" s="15" t="s">
+      <c r="K2" s="14" t="s">
         <v>8</v>
       </c>
       <c r="L2" s="1"/>
-      <c r="M2" s="14" t="s">
+      <c r="M2" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="N2" s="14" t="s">
+      <c r="N2" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="O2" s="14"/>
-      <c r="P2" s="14"/>
-      <c r="Q2" s="14"/>
-      <c r="R2" s="14"/>
-      <c r="S2" s="14"/>
-      <c r="T2" s="14" t="s">
+      <c r="O2" s="12"/>
+      <c r="P2" s="12"/>
+      <c r="Q2" s="12"/>
+      <c r="R2" s="12"/>
+      <c r="S2" s="12"/>
+      <c r="T2" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="U2" s="14" t="s">
+      <c r="U2" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="V2" s="16" t="s">
+      <c r="V2" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="W2" s="16" t="s">
+      <c r="W2" s="13" t="s">
         <v>13</v>
       </c>
       <c r="X2" s="2" t="s">
@@ -684,18 +691,18 @@
       </c>
     </row>
     <row r="3" spans="2:28" ht="45">
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="15"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="14"/>
       <c r="L3" s="1"/>
-      <c r="M3" s="14"/>
+      <c r="M3" s="12"/>
       <c r="N3" s="1" t="s">
         <v>15</v>
       </c>
@@ -714,10 +721,10 @@
       <c r="S3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="T3" s="14"/>
-      <c r="U3" s="14"/>
-      <c r="V3" s="16"/>
-      <c r="W3" s="16"/>
+      <c r="T3" s="12"/>
+      <c r="U3" s="12"/>
+      <c r="V3" s="13"/>
+      <c r="W3" s="13"/>
       <c r="X3" s="2"/>
     </row>
     <row r="4" spans="2:28">
@@ -738,13 +745,13 @@
         <v>0</v>
       </c>
       <c r="H4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I4" s="4">
         <v>25</v>
       </c>
       <c r="J4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K4" s="4">
         <v>3</v>
@@ -775,13 +782,13 @@
         <v>0</v>
       </c>
       <c r="H5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I5" s="4">
         <v>4</v>
       </c>
       <c r="J5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K5" s="4">
         <v>12</v>
@@ -812,13 +819,13 @@
         <v>0</v>
       </c>
       <c r="H6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I6" s="4">
         <v>1260</v>
       </c>
       <c r="J6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K6" s="4">
         <v>12</v>
@@ -851,13 +858,13 @@
         <v>0</v>
       </c>
       <c r="H7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I7" s="4">
         <v>86</v>
       </c>
       <c r="J7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K7" s="4">
         <v>3</v>
@@ -888,13 +895,13 @@
         <v>0</v>
       </c>
       <c r="H8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I8" s="4">
         <v>10</v>
       </c>
       <c r="J8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K8" s="4" t="s">
         <v>36</v>
@@ -923,13 +930,13 @@
         <v>0</v>
       </c>
       <c r="H9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I9" s="4">
         <v>1277</v>
       </c>
       <c r="J9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K9" s="4"/>
       <c r="N9" s="8" t="s">
@@ -1099,7 +1106,7 @@
     </row>
     <row r="14" spans="2:28">
       <c r="B14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D14">
         <v>15</v>
@@ -1115,22 +1122,25 @@
         <v>0</v>
       </c>
       <c r="H14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I14" s="4">
         <v>10</v>
       </c>
       <c r="J14" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K14" s="4">
-        <v>4</v>
+        <v>12</v>
+      </c>
+      <c r="L14">
+        <v>6</v>
       </c>
       <c r="M14" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N14" s="8" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="O14" s="9">
         <v>5</v>
@@ -1148,7 +1158,7 @@
         <v>14</v>
       </c>
       <c r="V14" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="W14" s="5">
         <v>95</v>
@@ -1156,8 +1166,8 @@
       <c r="X14" s="6"/>
     </row>
     <row r="15" spans="2:28">
-      <c r="B15" s="17" t="s">
-        <v>65</v>
+      <c r="B15" t="s">
+        <v>63</v>
       </c>
       <c r="D15">
         <v>16</v>
@@ -1167,31 +1177,31 @@
         <v>0x10</v>
       </c>
       <c r="F15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G15">
         <v>0</v>
       </c>
       <c r="H15" t="s">
+        <v>61</v>
+      </c>
+      <c r="I15" s="4">
+        <v>10</v>
+      </c>
+      <c r="J15" t="s">
         <v>62</v>
       </c>
-      <c r="I15" s="4">
-        <v>0</v>
-      </c>
-      <c r="J15" t="s">
-        <v>63</v>
-      </c>
       <c r="K15" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L15" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="M15" s="4">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N15" s="8" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="O15" s="9">
         <v>1</v>
@@ -1208,14 +1218,10 @@
       <c r="S15" s="9">
         <v>27</v>
       </c>
-      <c r="T15" s="4">
-        <v>10</v>
-      </c>
-      <c r="U15" s="4">
-        <v>2</v>
-      </c>
+      <c r="T15" s="16"/>
+      <c r="U15" s="16"/>
       <c r="V15" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="W15" s="5" t="s">
         <v>33</v>
@@ -1235,7 +1241,7 @@
         <v>0x11</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G16" s="11"/>
       <c r="H16" s="11"/>
@@ -1269,7 +1275,7 @@
         <v>0x14</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G17" s="11"/>
       <c r="H17" s="11"/>
@@ -1303,7 +1309,7 @@
         <v>0x15</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G18" s="11"/>
       <c r="H18" s="11"/>
@@ -1337,7 +1343,7 @@
         <v>0x16</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G19" s="11"/>
       <c r="H19" s="11"/>
@@ -1359,8 +1365,8 @@
       <c r="X19" s="6"/>
     </row>
     <row r="20" spans="2:24">
-      <c r="B20" s="12" t="s">
-        <v>57</v>
+      <c r="B20" s="16" t="s">
+        <v>56</v>
       </c>
       <c r="D20">
         <v>23</v>
@@ -1370,28 +1376,31 @@
         <v>0x17</v>
       </c>
       <c r="F20" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G20">
         <v>0</v>
       </c>
       <c r="H20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I20" s="4">
         <v>0</v>
       </c>
       <c r="J20" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K20" s="4">
         <v>2</v>
       </c>
+      <c r="L20">
+        <v>10</v>
+      </c>
       <c r="M20" s="4">
         <v>4</v>
       </c>
       <c r="N20" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O20" s="9">
         <v>0</v>
@@ -1415,7 +1424,7 @@
         <v>2</v>
       </c>
       <c r="V20" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="W20" s="5">
         <v>63</v>
@@ -1435,7 +1444,7 @@
         <v>0x18</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G21" s="11"/>
       <c r="H21" s="11"/>
@@ -1450,31 +1459,35 @@
       <c r="Q21" s="11"/>
       <c r="R21" s="11"/>
       <c r="S21" s="11"/>
-      <c r="T21" s="11"/>
-      <c r="U21" s="11"/>
+      <c r="T21" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="U21" s="17" t="s">
+        <v>69</v>
+      </c>
       <c r="V21" s="5"/>
       <c r="W21" s="5"/>
       <c r="X21" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:E3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:J3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="M2:M3"/>
     <mergeCell ref="N2:S2"/>
     <mergeCell ref="T2:T3"/>
     <mergeCell ref="U2:U3"/>
     <mergeCell ref="V2:V3"/>
     <mergeCell ref="W2:W3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:J3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:E3"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="G2:G3"/>
   </mergeCells>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>

</xml_diff>

<commit_message>
actualizacion en la funcion de calculate_register_units, unwrap podia suceder y generar panic, se arreglo con un unwrap_or, cambios en el match para el codigo de funcion 16, donde no se agregaban las count units o quantity units, se requiere tambien cambiar el tamaño de las Unit 1 en ProcessedTraces, ya que no eran sufientemente grandes por ser i16 y no u16 (no se alcanzaba el maximo u16 con i16) y tambien se ha implementado todo un bloque de tests, mediante trace_validation, falta las ultimas dos, read write y fifo queue a ser implementadas, por el momento pasan las pruebas pero deberia revisarle denuevo que las longitudes maximas no sea menores en las trazas, que creo haber olvidado
</commit_message>
<xml_diff>
--- a/modbus.xlsx
+++ b/modbus.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\windows\projects\rust\firerust\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75D2BCEE-3635-4434-8019-C151879B9C84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE6B7D9A-E605-4385-9341-A4EB4C479602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="74">
   <si>
     <t>MODBUS INSTRUCTION SAMPLE</t>
   </si>
@@ -258,6 +258,18 @@
   </si>
   <si>
     <t>pos 8 9</t>
+  </si>
+  <si>
+    <t>01 08 00 00 12 34 ED 7C</t>
+  </si>
+  <si>
+    <t>01 07 41 E2</t>
+  </si>
+  <si>
+    <t>01 0B 04 0A</t>
+  </si>
+  <si>
+    <t>01 0C 00 25</t>
   </si>
 </sst>
 </file>
@@ -339,7 +351,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -360,6 +372,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -372,8 +385,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -634,56 +645,56 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:28" ht="30" customHeight="1">
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="15"/>
-      <c r="F2" s="12" t="s">
+      <c r="E2" s="16"/>
+      <c r="F2" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="G2" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="12" t="s">
+      <c r="H2" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="14" t="s">
+      <c r="I2" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="12" t="s">
+      <c r="J2" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="K2" s="14" t="s">
+      <c r="K2" s="15" t="s">
         <v>8</v>
       </c>
       <c r="L2" s="1"/>
-      <c r="M2" s="12" t="s">
+      <c r="M2" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="N2" s="12" t="s">
+      <c r="N2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="O2" s="12"/>
-      <c r="P2" s="12"/>
-      <c r="Q2" s="12"/>
-      <c r="R2" s="12"/>
-      <c r="S2" s="12"/>
-      <c r="T2" s="12" t="s">
+      <c r="O2" s="13"/>
+      <c r="P2" s="13"/>
+      <c r="Q2" s="13"/>
+      <c r="R2" s="13"/>
+      <c r="S2" s="13"/>
+      <c r="T2" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="U2" s="12" t="s">
+      <c r="U2" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="V2" s="13" t="s">
+      <c r="V2" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="W2" s="13" t="s">
+      <c r="W2" s="14" t="s">
         <v>13</v>
       </c>
       <c r="X2" s="2" t="s">
@@ -691,18 +702,18 @@
       </c>
     </row>
     <row r="3" spans="2:28" ht="45">
-      <c r="B3" s="15"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="14"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="15"/>
       <c r="L3" s="1"/>
-      <c r="M3" s="12"/>
+      <c r="M3" s="13"/>
       <c r="N3" s="1" t="s">
         <v>15</v>
       </c>
@@ -721,10 +732,10 @@
       <c r="S3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="T3" s="12"/>
-      <c r="U3" s="12"/>
-      <c r="V3" s="13"/>
-      <c r="W3" s="13"/>
+      <c r="T3" s="13"/>
+      <c r="U3" s="13"/>
+      <c r="V3" s="14"/>
+      <c r="W3" s="14"/>
       <c r="X3" s="2"/>
     </row>
     <row r="4" spans="2:28">
@@ -742,7 +753,7 @@
         <v>22</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" t="s">
         <v>61</v>
@@ -779,7 +790,7 @@
         <v>26</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5" t="s">
         <v>61</v>
@@ -816,7 +827,7 @@
         <v>29</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6" t="s">
         <v>61</v>
@@ -855,7 +866,7 @@
         <v>32</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H7" t="s">
         <v>61</v>
@@ -892,7 +903,7 @@
         <v>35</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" t="s">
         <v>61</v>
@@ -927,7 +938,7 @@
         <v>39</v>
       </c>
       <c r="G9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9" t="s">
         <v>61</v>
@@ -970,7 +981,7 @@
     </row>
     <row r="10" spans="2:28">
       <c r="B10" s="10" t="s">
-        <v>43</v>
+        <v>71</v>
       </c>
       <c r="C10" s="10"/>
       <c r="D10" s="11">
@@ -1004,7 +1015,7 @@
     </row>
     <row r="11" spans="2:28">
       <c r="B11" s="11" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="C11" s="11"/>
       <c r="D11" s="11">
@@ -1038,7 +1049,7 @@
     </row>
     <row r="12" spans="2:28">
       <c r="B12" s="11" t="s">
-        <v>43</v>
+        <v>72</v>
       </c>
       <c r="C12" s="11"/>
       <c r="D12" s="11">
@@ -1072,7 +1083,7 @@
     </row>
     <row r="13" spans="2:28">
       <c r="B13" s="10" t="s">
-        <v>43</v>
+        <v>73</v>
       </c>
       <c r="C13" s="10"/>
       <c r="D13" s="11">
@@ -1119,7 +1130,7 @@
         <v>48</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14" t="s">
         <v>61</v>
@@ -1180,7 +1191,7 @@
         <v>50</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H15" t="s">
         <v>61</v>
@@ -1218,8 +1229,6 @@
       <c r="S15" s="9">
         <v>27</v>
       </c>
-      <c r="T15" s="16"/>
-      <c r="U15" s="16"/>
       <c r="V15" s="5" t="s">
         <v>51</v>
       </c>
@@ -1365,7 +1374,7 @@
       <c r="X19" s="6"/>
     </row>
     <row r="20" spans="2:24">
-      <c r="B20" s="16" t="s">
+      <c r="B20" t="s">
         <v>56</v>
       </c>
       <c r="D20">
@@ -1379,7 +1388,7 @@
         <v>57</v>
       </c>
       <c r="G20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H20" t="s">
         <v>61</v>
@@ -1459,10 +1468,10 @@
       <c r="Q21" s="11"/>
       <c r="R21" s="11"/>
       <c r="S21" s="11"/>
-      <c r="T21" s="17" t="s">
+      <c r="T21" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="U21" s="17" t="s">
+      <c r="U21" s="12" t="s">
         <v>69</v>
       </c>
       <c r="V21" s="5"/>

</xml_diff>